<commit_message>
Actualización proyecto Ampliación Mega
</commit_message>
<xml_diff>
--- a/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
+++ b/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
@@ -5,18 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/base de datos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/rigi-dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F639624F-9726-1949-8FBA-E1B8B4BC3652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6768F59F-1435-D647-9AC9-C083F6591518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36640" yWindow="600" windowWidth="32160" windowHeight="28200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36640" yWindow="600" windowWidth="32160" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyectos" sheetId="7" r:id="rId1"/>
     <sheet name="Diccionario" sheetId="6" r:id="rId2"/>
     <sheet name="Variable_Anterior" sheetId="8" r:id="rId3"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId4"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -98,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="483">
   <si>
     <t>id_proyecto</t>
   </si>
@@ -451,9 +454,6 @@
     <t>Rechazado</t>
   </si>
   <si>
-    <t>Mega</t>
-  </si>
-  <si>
     <t>Minera Agua Rica (MARA)</t>
   </si>
   <si>
@@ -1135,22 +1135,7 @@
     <t>https://www.geo-park.com/es/news/geopark-solicita-adhesion-al-rigi-por-proyecto-de-inversion/; https://econojournal.com.ar/oilgas/geopark-presenta-al-rigi-una-inversion-por-us1-000-millones-para-un-hub-petrolero-en-vaca-muerta/</t>
   </si>
   <si>
-    <t>Ampliación de la capacidad de procesamiento, fraccionamiento y transporte de líquidos del gas natural provenientes de la Cuenca Neuquina. Las obras abarcan instalaciones en Neuquén y el corredor de transporte hasta el complejo de fraccionamiento y exportación de Bahía Blanca, con un aumento proyectado de 1.500 toneladas diarias.</t>
-  </si>
-  <si>
     <t>YPF S.A. (Argentina); Petrobras (Brasil); Dow (Argentina)</t>
-  </si>
-  <si>
-    <t>Compañía Mega S.A. – Sucursal Dedicada</t>
-  </si>
-  <si>
-    <t>Neuquén; Río Negro; La Pampa; Buenos Aires</t>
-  </si>
-  <si>
-    <t>Globaris; EconoJournal; Compañía MEGA; Luis Caputo; auditoría 2026-08-08</t>
-  </si>
-  <si>
-    <t>https://econojournal.com.ar/oilgas/vaca-muerta-mega-se-presenta-al-rigi-con-una-inversion-de-us360-millones-en-su-planta-de-separacion-de-liquidos-del-gas/; https://www.ingenierowhite.com/2026/07/31/mega-obtuvo-la-aprobacion-de-su-proyecto-de-inversion-bajo-el-rigi/; https://x.com/LuisCaputoAR/status/2083255389399744911</t>
   </si>
   <si>
     <t>Desarrollo de una mina de cobre, oro, plata y molibdeno en Catamarca, integrando el yacimiento Agua Rica con la infraestructura existente de Alumbrera, ubicada a unos 35 km. El esquema MARA contempla explotación, procesamiento y uso de instalaciones compartidas para producción destinada principalmente a exportación.</t>
@@ -1557,14 +1542,45 @@
   <si>
     <t>Zijin Mining (China)</t>
   </si>
+  <si>
+    <t>Ampliación Mega</t>
+  </si>
+  <si>
+    <t>Ampliación de un complejo industrial para incrementar la capacidad de producción de Líquidos del Gas Natural (LGN) en 1500 toneladas diarias.  El proyecto contempla nuevas instalaciones en la Planta de Separación de Loma La Lata, la ampliación de la capacidad de transporte del poliducto que atraviesa Neuquén, Río Negro, La Pampa y Buenos Aires, y la expansión de la Planta de Fraccionamiento ubicada en Bahía Blanca.</t>
+  </si>
+  <si>
+    <t>Compañía Mega SA Sucursal Dedicada</t>
+  </si>
+  <si>
+    <t>30-71932893-4</t>
+  </si>
+  <si>
+    <t>Construcción de plantas de tratamiento, plantas de separación de líquidos de gas natural, oleoductos, gasoductos y poliductos e instalaciones de almacenamiento</t>
+  </si>
+  <si>
+    <t>Neuquén; La Pampa; Río Negro; Buenos Aires</t>
+  </si>
+  <si>
+    <t>Res. 1381/2026</t>
+  </si>
+  <si>
+    <t>La resolución define expresamente al proyecto como una ampliación de un proyecto preexistente no adherido al RIGI: el Complejo Industrial MEGA, cuya capacidad actual de producción de LGN será incrementada mediante nuevas instalaciones e infraestructura.</t>
+  </si>
+  <si>
+    <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/346397/20260826</t>
+  </si>
+  <si>
+    <t>Res. 1381/2026; Globaris; MECON</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -1720,7 +1736,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1804,6 +1820,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
@@ -2545,6 +2567,27 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Proyectos"/>
+      <sheetName val="Diccionario"/>
+      <sheetName val="Variable_Anterior"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Lucas Ordoñez" id="{3AB22868-5EC9-474A-BBCF-88B6CF007C82}" userId="aece5baeefa9fdd6" providerId="Windows Live"/>
@@ -2813,13 +2856,13 @@
   <sheetData>
     <row r="1" spans="1:30" ht="32">
       <c r="A1" s="23" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="D1" s="23" t="s">
         <v>0</v>
@@ -2828,10 +2871,10 @@
         <v>1</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G1" s="23" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="H1" s="23" t="s">
         <v>2</v>
@@ -2840,7 +2883,7 @@
         <v>3</v>
       </c>
       <c r="J1" s="23" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="K1" s="23" t="s">
         <v>4</v>
@@ -2849,69 +2892,69 @@
         <v>5</v>
       </c>
       <c r="M1" s="23" t="s">
+        <v>382</v>
+      </c>
+      <c r="N1" s="23" t="s">
+        <v>383</v>
+      </c>
+      <c r="O1" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="P1" s="23" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q1" s="23" t="s">
+        <v>386</v>
+      </c>
+      <c r="R1" s="23" t="s">
+        <v>387</v>
+      </c>
+      <c r="S1" s="23" t="s">
         <v>388</v>
       </c>
-      <c r="N1" s="23" t="s">
+      <c r="T1" s="23" t="s">
         <v>389</v>
       </c>
-      <c r="O1" s="23" t="s">
-        <v>390</v>
-      </c>
-      <c r="P1" s="23" t="s">
-        <v>391</v>
-      </c>
-      <c r="Q1" s="23" t="s">
-        <v>392</v>
-      </c>
-      <c r="R1" s="23" t="s">
-        <v>393</v>
-      </c>
-      <c r="S1" s="23" t="s">
-        <v>394</v>
-      </c>
-      <c r="T1" s="23" t="s">
-        <v>395</v>
-      </c>
       <c r="U1" s="23" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="V1" s="23" t="s">
         <v>6</v>
       </c>
       <c r="W1" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="X1" s="23" t="s">
         <v>156</v>
-      </c>
-      <c r="X1" s="23" t="s">
-        <v>157</v>
       </c>
       <c r="Y1" s="23" t="s">
         <v>7</v>
       </c>
       <c r="Z1" s="23" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="AA1" s="23" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="AB1" s="23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AC1" s="23" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="AD1" s="23" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="102">
       <c r="A2" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D2" s="6">
         <v>1</v>
@@ -2923,22 +2966,22 @@
         <v>9</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K2" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="M2" s="7">
         <v>550</v>
@@ -2981,16 +3024,16 @@
         <v>12</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AA2" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AB2" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AC2" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AD2" s="13"/>
     </row>
@@ -2999,10 +3042,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D3" s="14">
         <v>2</v>
@@ -3014,19 +3057,19 @@
         <v>17</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H3" s="15" t="s">
         <v>18</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K3" s="13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L3" s="13" t="s">
         <v>20</v>
@@ -3072,28 +3115,28 @@
         <v>21</v>
       </c>
       <c r="Z3" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA3" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AB3" s="18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC3" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AD3" s="13"/>
     </row>
     <row r="4" spans="1:30" ht="102">
       <c r="A4" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D4" s="6">
         <v>3</v>
@@ -3105,16 +3148,16 @@
         <v>23</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H4" s="15" t="s">
         <v>18</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K4" s="13" t="s">
         <v>24</v>
@@ -3163,16 +3206,16 @@
         <v>26</v>
       </c>
       <c r="Z4" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA4" s="13" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AB4" s="18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AC4" s="13" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AD4" s="13"/>
     </row>
@@ -3181,10 +3224,10 @@
         <v>27</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D5" s="14">
         <v>4</v>
@@ -3196,7 +3239,7 @@
         <v>29</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>10</v>
@@ -3254,16 +3297,16 @@
         <v>33</v>
       </c>
       <c r="Z5" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA5" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AB5" s="18" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AC5" s="13" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AD5" s="13"/>
     </row>
@@ -3272,28 +3315,28 @@
         <v>34</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="6">
         <v>5</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>10</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J6" s="5"/>
       <c r="K6" s="5" t="s">
@@ -3344,16 +3387,16 @@
         <v>37</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA6" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AB6" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AC6" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AD6" s="13"/>
     </row>
@@ -3362,10 +3405,10 @@
         <v>38</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D7" s="14">
         <v>6</v>
@@ -3374,19 +3417,19 @@
         <v>39</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>148</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>40</v>
@@ -3435,16 +3478,16 @@
         <v>41</v>
       </c>
       <c r="Z7" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA7" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AB7" s="19" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AC7" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AD7" s="13"/>
     </row>
@@ -3453,10 +3496,10 @@
         <v>42</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D8" s="6">
         <v>7</v>
@@ -3468,7 +3511,7 @@
         <v>44</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>45</v>
@@ -3477,7 +3520,7 @@
         <v>45</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>31</v>
@@ -3526,16 +3569,16 @@
         <v>46</v>
       </c>
       <c r="Z8" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA8" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AB8" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AC8" s="13" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AD8" s="13"/>
     </row>
@@ -3544,10 +3587,10 @@
         <v>47</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D9" s="14">
         <v>8</v>
@@ -3559,7 +3602,7 @@
         <v>49</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H9" s="7" t="s">
         <v>18</v>
@@ -3568,7 +3611,7 @@
         <v>50</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>36</v>
@@ -3617,28 +3660,28 @@
         <v>51</v>
       </c>
       <c r="Z9" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA9" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AB9" s="12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC9" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="AD9" s="13"/>
     </row>
     <row r="10" spans="1:30" ht="119">
       <c r="A10" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D10" s="6">
         <v>9</v>
@@ -3650,7 +3693,7 @@
         <v>53</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>18</v>
@@ -3659,7 +3702,7 @@
         <v>54</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K10" s="13" t="s">
         <v>19</v>
@@ -3708,28 +3751,28 @@
         <v>55</v>
       </c>
       <c r="Z10" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AA10" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AB10" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AC10" s="13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AD10" s="13"/>
     </row>
     <row r="11" spans="1:30" ht="255">
       <c r="A11" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D11" s="14">
         <v>10</v>
@@ -3738,10 +3781,10 @@
         <v>52</v>
       </c>
       <c r="F11" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>193</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>194</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>18</v>
@@ -3750,7 +3793,7 @@
         <v>54</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>56</v>
@@ -3799,28 +3842,28 @@
         <v>57</v>
       </c>
       <c r="Z11" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AA11" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AB11" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AC11" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AD11" s="13"/>
     </row>
     <row r="12" spans="1:30" ht="119">
       <c r="A12" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D12" s="6">
         <v>11</v>
@@ -3832,7 +3875,7 @@
         <v>59</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>60</v>
@@ -3841,7 +3884,7 @@
         <v>61</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="K12" s="5" t="s">
         <v>62</v>
@@ -3890,28 +3933,28 @@
         <v>63</v>
       </c>
       <c r="Z12" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA12" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AB12" s="12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AC12" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AD12" s="13"/>
     </row>
     <row r="13" spans="1:30" ht="372">
       <c r="A13" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D13" s="14">
         <v>12</v>
@@ -3923,16 +3966,16 @@
         <v>65</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K13" s="13" t="s">
         <v>40</v>
@@ -3981,28 +4024,28 @@
         <v>66</v>
       </c>
       <c r="Z13" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA13" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AB13" s="18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AC13" s="13" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AD13" s="13"/>
     </row>
     <row r="14" spans="1:30" ht="136">
       <c r="A14" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D14" s="6">
         <v>13</v>
@@ -4011,19 +4054,19 @@
         <v>67</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>18</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K14" s="5" t="s">
         <v>24</v>
@@ -4072,16 +4115,16 @@
         <v>68</v>
       </c>
       <c r="Z14" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AA14" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AB14" s="12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AC14" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AD14" s="13"/>
     </row>
@@ -4090,17 +4133,17 @@
         <v>76</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="14">
         <v>14</v>
       </c>
       <c r="E15" s="28" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G15" s="13"/>
       <c r="H15" s="15" t="s">
@@ -4130,7 +4173,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T15" s="13"/>
       <c r="U15" s="10"/>
@@ -4144,10 +4187,10 @@
       <c r="AA15" s="13"/>
       <c r="AB15" s="13"/>
       <c r="AC15" s="13" t="s">
+        <v>299</v>
+      </c>
+      <c r="AD15" s="13" t="s">
         <v>300</v>
-      </c>
-      <c r="AD15" s="13" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="16" spans="1:30" ht="409.6">
@@ -4155,7 +4198,7 @@
         <v>77</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="6">
@@ -4195,7 +4238,7 @@
         <v>0</v>
       </c>
       <c r="S16" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T16" s="5"/>
       <c r="U16" s="10"/>
@@ -4209,10 +4252,10 @@
       <c r="AA16" s="5"/>
       <c r="AB16" s="5"/>
       <c r="AC16" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="AD16" s="13" t="s">
         <v>303</v>
-      </c>
-      <c r="AD16" s="13" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="17" spans="1:30" ht="409.6">
@@ -4220,24 +4263,24 @@
         <v>81</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="14">
         <v>16</v>
       </c>
       <c r="E17" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="F17" s="13" t="s">
         <v>306</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>307</v>
       </c>
       <c r="G17" s="13"/>
       <c r="H17" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="s">
@@ -4260,7 +4303,7 @@
         <v>0</v>
       </c>
       <c r="S17" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T17" s="13"/>
       <c r="U17" s="10"/>
@@ -4274,21 +4317,21 @@
       <c r="AA17" s="13"/>
       <c r="AB17" s="13"/>
       <c r="AC17" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="AD17" s="13" t="s">
         <v>309</v>
-      </c>
-      <c r="AD17" s="13" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="18" spans="1:30" ht="119">
       <c r="A18" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D18" s="6">
         <v>17</v>
@@ -4297,10 +4340,10 @@
         <v>83</v>
       </c>
       <c r="F18" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>200</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>201</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>18</v>
@@ -4309,7 +4352,7 @@
         <v>54</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K18" s="5" t="s">
         <v>84</v>
@@ -4355,19 +4398,19 @@
         <v>46177</v>
       </c>
       <c r="Y18" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="Z18" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="AA18" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="AB18" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="Z18" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="AA18" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="AB18" s="12" t="s">
-        <v>203</v>
-      </c>
       <c r="AC18" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AD18" s="13"/>
     </row>
@@ -4376,7 +4419,7 @@
         <v>85</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="14">
@@ -4390,14 +4433,14 @@
       </c>
       <c r="G19" s="13"/>
       <c r="H19" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J19" s="13"/>
       <c r="K19" s="13" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="L19" s="13" t="s">
         <v>11</v>
@@ -4416,7 +4459,7 @@
         <v>0</v>
       </c>
       <c r="S19" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T19" s="13"/>
       <c r="U19" s="10"/>
@@ -4430,10 +4473,10 @@
       <c r="AA19" s="13"/>
       <c r="AB19" s="13"/>
       <c r="AC19" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="AD19" s="13" t="s">
         <v>313</v>
-      </c>
-      <c r="AD19" s="13" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="20" spans="1:30" ht="409.6">
@@ -4441,7 +4484,7 @@
         <v>88</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="6">
@@ -4481,7 +4524,7 @@
         <v>0</v>
       </c>
       <c r="S20" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T20" s="5"/>
       <c r="U20" s="10"/>
@@ -4495,10 +4538,10 @@
       <c r="AA20" s="5"/>
       <c r="AB20" s="5"/>
       <c r="AC20" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="AD20" s="13" t="s">
         <v>316</v>
-      </c>
-      <c r="AD20" s="13" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="21" spans="1:30" ht="409.6">
@@ -4506,7 +4549,7 @@
         <v>91</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="14">
@@ -4516,14 +4559,14 @@
         <v>92</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="G21" s="13"/>
       <c r="H21" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J21" s="13"/>
       <c r="K21" s="13" t="s">
@@ -4546,7 +4589,7 @@
         <v>0</v>
       </c>
       <c r="S21" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T21" s="13"/>
       <c r="U21" s="10"/>
@@ -4560,10 +4603,10 @@
       <c r="AA21" s="13"/>
       <c r="AB21" s="13"/>
       <c r="AC21" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="AD21" s="13" t="s">
         <v>319</v>
-      </c>
-      <c r="AD21" s="13" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="22" spans="1:30" ht="409.6">
@@ -4571,17 +4614,17 @@
         <v>93</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="6">
         <v>21</v>
       </c>
       <c r="E22" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>322</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>323</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="7" t="s">
@@ -4592,10 +4635,10 @@
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="L22" s="5" t="s">
         <v>324</v>
-      </c>
-      <c r="L22" s="5" t="s">
-        <v>325</v>
       </c>
       <c r="M22" s="7">
         <v>200</v>
@@ -4611,7 +4654,7 @@
         <v>0</v>
       </c>
       <c r="S22" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T22" s="5"/>
       <c r="U22" s="10"/>
@@ -4625,10 +4668,10 @@
       <c r="AA22" s="5"/>
       <c r="AB22" s="5"/>
       <c r="AC22" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="AD22" s="13" t="s">
         <v>326</v>
-      </c>
-      <c r="AD22" s="13" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="23" spans="1:30" ht="409.6">
@@ -4636,7 +4679,7 @@
         <v>95</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="14">
@@ -4676,7 +4719,7 @@
         <v>0</v>
       </c>
       <c r="S23" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T23" s="13"/>
       <c r="U23" s="10"/>
@@ -4690,10 +4733,10 @@
       <c r="AA23" s="13"/>
       <c r="AB23" s="13"/>
       <c r="AC23" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="AD23" s="13" t="s">
         <v>329</v>
-      </c>
-      <c r="AD23" s="13" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="24" spans="1:30" ht="409.6">
@@ -4701,7 +4744,7 @@
         <v>98</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="6">
@@ -4715,10 +4758,10 @@
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="5" t="s">
@@ -4741,7 +4784,7 @@
         <v>0</v>
       </c>
       <c r="S24" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T24" s="5"/>
       <c r="U24" s="10"/>
@@ -4755,10 +4798,10 @@
       <c r="AA24" s="5"/>
       <c r="AB24" s="5"/>
       <c r="AC24" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="AD24" s="13" t="s">
         <v>332</v>
-      </c>
-      <c r="AD24" s="13" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="25" spans="1:30" ht="409.6">
@@ -4766,14 +4809,14 @@
         <v>101</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C25" s="13"/>
       <c r="D25" s="14">
         <v>24</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>102</v>
@@ -4806,7 +4849,7 @@
         <v>0</v>
       </c>
       <c r="S25" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T25" s="13"/>
       <c r="U25" s="10"/>
@@ -4820,21 +4863,21 @@
       <c r="AA25" s="13"/>
       <c r="AB25" s="13"/>
       <c r="AC25" s="13" t="s">
+        <v>335</v>
+      </c>
+      <c r="AD25" s="13" t="s">
         <v>336</v>
-      </c>
-      <c r="AD25" s="13" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="26" spans="1:30" ht="289">
       <c r="A26" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D26" s="6">
         <v>25</v>
@@ -4846,16 +4889,16 @@
         <v>104</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="K26" s="5" t="s">
         <v>82</v>
@@ -4901,31 +4944,31 @@
         <v>46224</v>
       </c>
       <c r="Y26" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Z26" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AA26" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="AB26" s="12" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="AC26" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AD26" s="13"/>
     </row>
     <row r="27" spans="1:30" ht="255">
       <c r="A27" s="13" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D27" s="14">
         <v>26</v>
@@ -4934,10 +4977,10 @@
         <v>105</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>18</v>
@@ -4946,10 +4989,10 @@
         <v>54</v>
       </c>
       <c r="J27" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K27" s="13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L27" s="13" t="s">
         <v>20</v>
@@ -4992,19 +5035,19 @@
         <v>46234</v>
       </c>
       <c r="Y27" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="Z27" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AA27" s="13" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="AB27" s="21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="AC27" s="13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="AD27" s="13"/>
     </row>
@@ -5013,7 +5056,7 @@
         <v>106</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="6">
@@ -5053,7 +5096,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T28" s="5"/>
       <c r="U28" s="10"/>
@@ -5067,31 +5110,31 @@
       <c r="AA28" s="5"/>
       <c r="AB28" s="5"/>
       <c r="AC28" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="AD28" s="13" t="s">
         <v>339</v>
-      </c>
-      <c r="AD28" s="13" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="29" spans="1:30" ht="289">
       <c r="A29" s="13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C29" s="13"/>
       <c r="D29" s="14">
         <v>28</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="F29" s="13" t="s">
         <v>108</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>18</v>
@@ -5100,7 +5143,7 @@
         <v>54</v>
       </c>
       <c r="J29" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K29" s="13" t="s">
         <v>56</v>
@@ -5146,19 +5189,19 @@
         <v>46232</v>
       </c>
       <c r="Y29" s="13" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="Z29" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AA29" s="13" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AB29" s="18" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AC29" s="13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="AD29" s="13"/>
     </row>
@@ -5167,10 +5210,10 @@
         <v>109</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D30" s="6">
         <v>29</v>
@@ -5182,16 +5225,16 @@
         <v>111</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="H30" s="7" t="s">
         <v>18</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>24</v>
@@ -5238,19 +5281,19 @@
         <v>46233</v>
       </c>
       <c r="Y30" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="Z30" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="AA30" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="AB30" s="12" t="s">
         <v>278</v>
       </c>
-      <c r="Z30" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="AA30" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="AB30" s="12" t="s">
+      <c r="AC30" s="5" t="s">
         <v>279</v>
-      </c>
-      <c r="AC30" s="5" t="s">
-        <v>280</v>
       </c>
       <c r="AD30" s="13"/>
     </row>
@@ -5259,24 +5302,24 @@
         <v>112</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="14">
         <v>30</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F31" s="22" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J31" s="5"/>
       <c r="K31" s="5" t="s">
@@ -5299,7 +5342,7 @@
         <v>0</v>
       </c>
       <c r="S31" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T31" s="5"/>
       <c r="U31" s="10"/>
@@ -5313,21 +5356,21 @@
       <c r="AA31" s="5"/>
       <c r="AB31" s="5"/>
       <c r="AC31" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="AD31" s="13" t="s">
         <v>343</v>
-      </c>
-      <c r="AD31" s="13" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="32" spans="1:30" ht="119">
       <c r="A32" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>160</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>161</v>
       </c>
       <c r="D32" s="6">
         <v>31</v>
@@ -5339,7 +5382,7 @@
         <v>74</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H32" s="7" t="s">
         <v>18</v>
@@ -5348,7 +5391,7 @@
         <v>50</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>24</v>
@@ -5397,16 +5440,16 @@
         <v>75</v>
       </c>
       <c r="Z32" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AA32" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AB32" s="12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AC32" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="AD32" s="13"/>
     </row>
@@ -5467,81 +5510,107 @@
       <c r="AA33" s="13"/>
       <c r="AB33" s="13"/>
       <c r="AC33" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AD33" s="13"/>
     </row>
-    <row r="34" spans="1:30" ht="409.6">
-      <c r="A34" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="C34" s="5"/>
-      <c r="D34" s="6">
+    <row r="34" spans="1:30" ht="136">
+      <c r="A34" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="D34" s="14">
         <v>33</v>
       </c>
-      <c r="E34" s="7" t="s">
-        <v>346</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="G34" s="5"/>
-      <c r="H34" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="I34" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5" t="s">
-        <v>348</v>
+      <c r="E34" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>475</v>
+      </c>
+      <c r="G34" s="13" t="s">
+        <v>476</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="I34" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="J34" s="13" t="s">
+        <v>477</v>
+      </c>
+      <c r="K34" s="13" t="s">
+        <v>478</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="M34" s="7">
-        <v>360</v>
-      </c>
-      <c r="N34" s="7">
-        <v>360</v>
-      </c>
-      <c r="O34" s="7"/>
-      <c r="P34" s="8"/>
-      <c r="Q34" s="8"/>
-      <c r="R34" s="9">
-        <f>SUM(Tabla22[[#This Row],[inversion_activos_computables_comprometida_anio_1_mill_usd]:[inversion_activos_computables_comprometida_anio_2_mill_usd]])</f>
-        <v>0</v>
-      </c>
-      <c r="S34" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="T34" s="5"/>
-      <c r="U34" s="10"/>
-      <c r="V34" s="11">
+        <v>324</v>
+      </c>
+      <c r="M34" s="29">
+        <v>365.39866899999998</v>
+      </c>
+      <c r="N34" s="29">
+        <v>365.39866899999998</v>
+      </c>
+      <c r="O34" s="15">
+        <v>359.16436099999999</v>
+      </c>
+      <c r="P34" s="16">
+        <v>121.613889</v>
+      </c>
+      <c r="Q34" s="16">
+        <v>152.70910599999999</v>
+      </c>
+      <c r="R34" s="16">
+        <f>SUM([1]!Tabla22[[#This Row],[inversion_activos_computables_comprometida_anio_1_mill_usd]:[inversion_activos_computables_comprometida_anio_2_mill_usd]])</f>
+        <v>274.32299499999999</v>
+      </c>
+      <c r="S34" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="T34" s="15">
+        <v>792</v>
+      </c>
+      <c r="U34" s="30">
+        <v>46661</v>
+      </c>
+      <c r="V34" s="17">
         <v>46099</v>
       </c>
-      <c r="W34" s="11"/>
-      <c r="X34" s="11"/>
-      <c r="Y34" s="5"/>
-      <c r="Z34" s="5"/>
-      <c r="AA34" s="5"/>
-      <c r="AB34" s="5"/>
-      <c r="AC34" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="AD34" s="13" t="s">
-        <v>350</v>
-      </c>
+      <c r="W34" s="17">
+        <v>46231</v>
+      </c>
+      <c r="X34" s="17">
+        <v>46260</v>
+      </c>
+      <c r="Y34" s="13" t="s">
+        <v>479</v>
+      </c>
+      <c r="Z34" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="AA34" s="13" t="s">
+        <v>480</v>
+      </c>
+      <c r="AB34" s="13" t="s">
+        <v>481</v>
+      </c>
+      <c r="AC34" s="13" t="s">
+        <v>482</v>
+      </c>
+      <c r="AD34" s="13"/>
     </row>
     <row r="35" spans="1:30" ht="409.6">
       <c r="A35" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="C35" s="13"/>
       <c r="D35" s="14">
@@ -5551,7 +5620,7 @@
         <v>89</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G35" s="13"/>
       <c r="H35" s="15" t="s">
@@ -5581,7 +5650,7 @@
         <v>0</v>
       </c>
       <c r="S35" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T35" s="13"/>
       <c r="U35" s="10"/>
@@ -5595,18 +5664,18 @@
       <c r="AA35" s="13"/>
       <c r="AB35" s="13"/>
       <c r="AC35" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="AD35" s="13" t="s">
         <v>316</v>
-      </c>
-      <c r="AD35" s="13" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="36" spans="1:30" ht="409.6">
       <c r="A36" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="6">
@@ -5616,14 +5685,14 @@
         <v>103</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G36" s="5"/>
       <c r="H36" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="5" t="s">
@@ -5646,7 +5715,7 @@
         <v>0</v>
       </c>
       <c r="S36" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T36" s="5"/>
       <c r="U36" s="10"/>
@@ -5660,45 +5729,45 @@
       <c r="AA36" s="5"/>
       <c r="AB36" s="5"/>
       <c r="AC36" s="5" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="AD36" s="13" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
     </row>
     <row r="37" spans="1:30" ht="204">
       <c r="A37" s="13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D37" s="14">
         <v>36</v>
       </c>
       <c r="E37" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="F37" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="F37" s="13" t="s">
-        <v>123</v>
-      </c>
       <c r="G37" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="I37" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="J37" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="K37" s="13" t="s">
         <v>242</v>
-      </c>
-      <c r="H37" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="I37" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="J37" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="K37" s="13" t="s">
-        <v>243</v>
       </c>
       <c r="L37" s="13" t="s">
         <v>11</v>
@@ -5741,19 +5810,19 @@
         <v>46198</v>
       </c>
       <c r="Y37" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="Z37" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="AA37" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="AB37" s="21" t="s">
         <v>244</v>
       </c>
-      <c r="Z37" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="AA37" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="AB37" s="21" t="s">
+      <c r="AC37" s="13" t="s">
         <v>245</v>
-      </c>
-      <c r="AC37" s="13" t="s">
-        <v>246</v>
       </c>
       <c r="AD37" s="13"/>
     </row>
@@ -5762,10 +5831,10 @@
         <v>69</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D38" s="6">
         <v>37</v>
@@ -5777,7 +5846,7 @@
         <v>71</v>
       </c>
       <c r="G38" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H38" s="15" t="s">
         <v>18</v>
@@ -5786,7 +5855,7 @@
         <v>54</v>
       </c>
       <c r="J38" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K38" s="13" t="s">
         <v>56</v>
@@ -5835,35 +5904,35 @@
         <v>72</v>
       </c>
       <c r="Z38" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AA38" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AB38" s="21" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AC38" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="AD38" s="13"/>
     </row>
     <row r="39" spans="1:30" ht="409.6">
       <c r="A39" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="14">
         <v>38</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="G39" s="5"/>
       <c r="H39" s="7" t="s">
@@ -5893,7 +5962,7 @@
         <v>0</v>
       </c>
       <c r="S39" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T39" s="5"/>
       <c r="U39" s="10"/>
@@ -5907,35 +5976,35 @@
       <c r="AA39" s="5"/>
       <c r="AB39" s="5"/>
       <c r="AC39" s="5" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="AD39" s="13" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
     </row>
     <row r="40" spans="1:30" ht="409.6">
       <c r="A40" s="13" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="6">
         <v>39</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="G40" s="13"/>
       <c r="H40" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I40" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J40" s="13"/>
       <c r="K40" s="13" t="s">
@@ -5958,7 +6027,7 @@
         <v>0</v>
       </c>
       <c r="S40" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T40" s="13"/>
       <c r="U40" s="10"/>
@@ -5972,35 +6041,35 @@
       <c r="AA40" s="13"/>
       <c r="AB40" s="13"/>
       <c r="AC40" s="13" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="AD40" s="13" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
     </row>
     <row r="41" spans="1:30" ht="409.6">
       <c r="A41" s="13" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="C41" s="13"/>
       <c r="D41" s="14">
         <v>40</v>
       </c>
       <c r="E41" s="15" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="G41" s="13"/>
       <c r="H41" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I41" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J41" s="13"/>
       <c r="K41" s="13" t="s">
@@ -6023,7 +6092,7 @@
         <v>0</v>
       </c>
       <c r="S41" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T41" s="17"/>
       <c r="U41" s="10"/>
@@ -6037,39 +6106,39 @@
       <c r="AA41" s="13"/>
       <c r="AB41" s="13"/>
       <c r="AC41" s="13" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
       <c r="AD41" s="18" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
     </row>
     <row r="42" spans="1:30" ht="409.6">
       <c r="A42" s="13" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="14">
         <v>41</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="G42" s="13"/>
       <c r="H42" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I42" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J42" s="13"/>
       <c r="K42" s="13" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="L42" s="13" t="s">
         <v>11</v>
@@ -6086,7 +6155,7 @@
         <v>0</v>
       </c>
       <c r="S42" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T42" s="15"/>
       <c r="U42" s="10"/>
@@ -6100,10 +6169,10 @@
       <c r="AA42" s="13"/>
       <c r="AB42" s="13"/>
       <c r="AC42" s="13" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="AD42" s="13" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
     </row>
     <row r="43" spans="1:30">
@@ -6188,22 +6257,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="24" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="C1" s="24" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16">
@@ -6211,19 +6280,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16">
@@ -6231,19 +6300,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16">
@@ -6251,19 +6320,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16">
@@ -6274,16 +6343,16 @@
         <v>0</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16">
@@ -6294,16 +6363,16 @@
         <v>1</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16">
@@ -6311,19 +6380,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16">
@@ -6331,19 +6400,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16">
@@ -6354,16 +6423,16 @@
         <v>2</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16">
@@ -6374,16 +6443,16 @@
         <v>3</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16">
@@ -6391,19 +6460,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16">
@@ -6414,16 +6483,16 @@
         <v>4</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16">
@@ -6434,16 +6503,16 @@
         <v>5</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16">
@@ -6451,19 +6520,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16">
@@ -6471,19 +6540,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16">
@@ -6491,19 +6560,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="D16" s="23" t="s">
+        <v>429</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>430</v>
+      </c>
+      <c r="F16" s="23" t="s">
         <v>435</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>436</v>
-      </c>
-      <c r="F16" s="23" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="16">
@@ -6511,19 +6580,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="16">
@@ -6531,19 +6600,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="32">
@@ -6551,19 +6620,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="16">
@@ -6571,19 +6640,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F20" s="23" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16">
@@ -6591,19 +6660,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="16">
@@ -6611,19 +6680,19 @@
         <v>21</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="16">
@@ -6634,16 +6703,16 @@
         <v>6</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="16">
@@ -6651,19 +6720,19 @@
         <v>23</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="16">
@@ -6671,19 +6740,19 @@
         <v>24</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="16">
@@ -6694,16 +6763,16 @@
         <v>7</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="32">
@@ -6711,19 +6780,19 @@
         <v>26</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="16">
@@ -6731,19 +6800,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="16">
@@ -6751,19 +6820,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="16">
@@ -6771,19 +6840,19 @@
         <v>29</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="16">
@@ -6791,19 +6860,19 @@
         <v>30</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
     </row>
   </sheetData>
@@ -6818,13 +6887,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="60">
       <c r="A1" s="26" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -6832,10 +6901,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="45">
@@ -6843,10 +6912,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="105">
@@ -6854,10 +6923,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -6887,10 +6956,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -6898,10 +6967,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -6931,10 +7000,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -6964,10 +7033,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="60">
@@ -6975,10 +7044,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="60">
@@ -6986,10 +7055,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="90">
@@ -6997,10 +7066,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="90">
@@ -7008,10 +7077,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="90">
@@ -7019,10 +7088,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="45">
@@ -7030,10 +7099,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="60">
@@ -7041,10 +7110,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="75">
@@ -7052,10 +7121,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30">
@@ -7074,10 +7143,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30">
@@ -7085,10 +7154,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="30">
@@ -7107,10 +7176,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="27" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="60">
@@ -7118,10 +7187,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -7129,10 +7198,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="27" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -7140,10 +7209,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="27" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="30">
@@ -7151,10 +7220,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualización proyecto fertilizantes 7/09/2026
</commit_message>
<xml_diff>
--- a/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
+++ b/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/rigi-dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6768F59F-1435-D647-9AC9-C083F6591518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70E72C1D-546E-0546-819C-35C80583B28D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="36640" yWindow="600" windowWidth="32160" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="487">
   <si>
     <t>id_proyecto</t>
   </si>
@@ -460,9 +460,6 @@
     <t>Minera Agua Rica LLC Sucursal Argentina</t>
   </si>
   <si>
-    <t>Fértil Pampa</t>
-  </si>
-  <si>
     <t>Fértil Pampa S.A.U.</t>
   </si>
   <si>
@@ -1139,18 +1136,6 @@
   </si>
   <si>
     <t>Desarrollo de una mina de cobre, oro, plata y molibdeno en Catamarca, integrando el yacimiento Agua Rica con la infraestructura existente de Alumbrera, ubicada a unos 35 km. El esquema MARA contempla explotación, procesamiento y uso de instalaciones compartidas para producción destinada principalmente a exportación.</t>
-  </si>
-  <si>
-    <t>Construcción de un complejo industrial de amoníaco y urea granulada en Bahía Blanca, provincia de Buenos Aires, a cargo de Fértil Pampa. La planta tendrá dos trenes de urea, instalaciones auxiliares, almacenamiento y logística portuaria, con capacidad prevista de 2,1 millones de toneladas anuales.</t>
-  </si>
-  <si>
-    <t>Petroquímica / Fertilizantes</t>
-  </si>
-  <si>
-    <t>Globaris; Pampa Energía; International Finance Corporation; El Cronista; La Nación; Luis Caputo; auditoría 2026-08-08</t>
-  </si>
-  <si>
-    <t>https://ri.pampa.com/en/press-release/pampa-energia-announces-its-entry-into-the-fertilizer-business-with-the-construction-of-latin-americas-largest-urea-plant/; https://disclosures.ifc.org/project-detail/ED/52106/fer-il-p; https://www.cronista.com/negocios/fertil-pampa-se-presenta-al-rigi-con-una-inversion-de-us-2400-millones-para-producir-fertilizantes/; https://www.lanacion.com.ar/economia/campo/invertiria-us2400-millones-una-empresa-de-marcelo-mindlin-pidio-ingresar-al-rigi-para-producir-nid23042026/</t>
   </si>
   <si>
     <t>Desarrollo integrado de litio en los proyectos Jama y Solaroz, en la Puna de Jujuy, con una planta prevista en el Salar de Jama. La iniciativa contempla extracción de salmuera y producción de compuestos de litio, con una capacidad informada de aproximadamente 22.000 toneladas anuales.</t>
@@ -1572,6 +1557,33 @@
   <si>
     <t>Res. 1381/2026; Globaris; MECON</t>
   </si>
+  <si>
+    <t>Fertilizantes</t>
+  </si>
+  <si>
+    <t>Construcción, operación y gerenciamiento de dos (2) plantas de producción de urea, cada una con capacidad de tres mil toneladas (3.000 t) por día, con sus correspondientes unidades de granulación, y una planta de amoníaco con capacidad de tres mil cuatrocientas cincuenta toneladas (3.450 t) por día, utilizando como insumo principal el gas natural de Vaca Muerta, a desarrollarse en el Puerto de Ingeniero White, partido de Bahía Blanca, provincia de Buenos Aires.</t>
+  </si>
+  <si>
+    <t>30-71875855-2</t>
+  </si>
+  <si>
+    <t>Petroquímica y Fertilizantes</t>
+  </si>
+  <si>
+    <t>Puerto de Ingeniero White, Bahía Blanca</t>
+  </si>
+  <si>
+    <t>Res. 1468/2026</t>
+  </si>
+  <si>
+    <t>Se identifican signos fuertes de preexistencia. El proyecto “Fertilizantes” de Fértil Pampa SAU fue aprobado bajo RIGI por la Resolución 1468/2026, publicada el 07/09/2026, pero existía públicamente antes de esa fecha. La sociedad Fértil Pampa SAU fue constituida en octubre de 2024 con objeto específico de construir y operar una planta de amoníaco, urea y otros fertilizantes. Antes de la aprobación RIGI ya existían divulgaciones financieras y ambientales ante BID Invest e IFC, solicitud RIGI presentada el 21/04/2026, memorándum de entendimiento con el Municipio de Bahía Blanca, decisión final de inversión de Pampa Energía del 17/07/2026, contrato EPC con Tecnimont–SACDE y trámites de participación pública ambiental. Por lo tanto, se clasifica como proyecto preexistente al anuncio/aprobación oficial, aunque corresponde a una inversión greenfield y no a una ampliación de una planta ya operativa.</t>
+  </si>
+  <si>
+    <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/346966/20260907</t>
+  </si>
+  <si>
+    <t>Res.1468/2026; MECON</t>
+  </si>
 </sst>
 </file>
 
@@ -1582,7 +1594,7 @@
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1668,6 +1680,13 @@
       <color rgb="FF000000"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1736,7 +1755,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1824,6 +1843,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2856,13 +2881,13 @@
   <sheetData>
     <row r="1" spans="1:30" ht="32">
       <c r="A1" s="23" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="D1" s="23" t="s">
         <v>0</v>
@@ -2871,10 +2896,10 @@
         <v>1</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G1" s="23" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="H1" s="23" t="s">
         <v>2</v>
@@ -2883,7 +2908,7 @@
         <v>3</v>
       </c>
       <c r="J1" s="23" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="K1" s="23" t="s">
         <v>4</v>
@@ -2892,69 +2917,69 @@
         <v>5</v>
       </c>
       <c r="M1" s="23" t="s">
+        <v>377</v>
+      </c>
+      <c r="N1" s="23" t="s">
+        <v>378</v>
+      </c>
+      <c r="O1" s="23" t="s">
+        <v>379</v>
+      </c>
+      <c r="P1" s="23" t="s">
+        <v>380</v>
+      </c>
+      <c r="Q1" s="23" t="s">
+        <v>381</v>
+      </c>
+      <c r="R1" s="23" t="s">
         <v>382</v>
       </c>
-      <c r="N1" s="23" t="s">
+      <c r="S1" s="23" t="s">
         <v>383</v>
       </c>
-      <c r="O1" s="23" t="s">
+      <c r="T1" s="23" t="s">
         <v>384</v>
       </c>
-      <c r="P1" s="23" t="s">
-        <v>385</v>
-      </c>
-      <c r="Q1" s="23" t="s">
-        <v>386</v>
-      </c>
-      <c r="R1" s="23" t="s">
-        <v>387</v>
-      </c>
-      <c r="S1" s="23" t="s">
-        <v>388</v>
-      </c>
-      <c r="T1" s="23" t="s">
-        <v>389</v>
-      </c>
       <c r="U1" s="23" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="V1" s="23" t="s">
         <v>6</v>
       </c>
       <c r="W1" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="X1" s="23" t="s">
         <v>155</v>
-      </c>
-      <c r="X1" s="23" t="s">
-        <v>156</v>
       </c>
       <c r="Y1" s="23" t="s">
         <v>7</v>
       </c>
       <c r="Z1" s="23" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="AA1" s="23" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="AB1" s="23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AC1" s="23" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="AD1" s="23" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="102">
       <c r="A2" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D2" s="6">
         <v>1</v>
@@ -2966,22 +2991,22 @@
         <v>9</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K2" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>175</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>176</v>
       </c>
       <c r="M2" s="7">
         <v>550</v>
@@ -3024,16 +3049,16 @@
         <v>12</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AA2" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AB2" s="12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AC2" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AD2" s="13"/>
     </row>
@@ -3042,10 +3067,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D3" s="14">
         <v>2</v>
@@ -3057,19 +3082,19 @@
         <v>17</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H3" s="15" t="s">
         <v>18</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K3" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L3" s="13" t="s">
         <v>20</v>
@@ -3115,28 +3140,28 @@
         <v>21</v>
       </c>
       <c r="Z3" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA3" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AB3" s="18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AC3" s="13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AD3" s="13"/>
     </row>
     <row r="4" spans="1:30" ht="102">
       <c r="A4" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D4" s="6">
         <v>3</v>
@@ -3148,16 +3173,16 @@
         <v>23</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H4" s="15" t="s">
         <v>18</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K4" s="13" t="s">
         <v>24</v>
@@ -3206,16 +3231,16 @@
         <v>26</v>
       </c>
       <c r="Z4" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA4" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AB4" s="18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC4" s="13" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="AD4" s="13"/>
     </row>
@@ -3224,10 +3249,10 @@
         <v>27</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D5" s="14">
         <v>4</v>
@@ -3239,7 +3264,7 @@
         <v>29</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>10</v>
@@ -3297,16 +3322,16 @@
         <v>33</v>
       </c>
       <c r="Z5" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA5" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AB5" s="18" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AC5" s="13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AD5" s="13"/>
     </row>
@@ -3315,28 +3340,28 @@
         <v>34</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D6" s="6">
         <v>5</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>10</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J6" s="5"/>
       <c r="K6" s="5" t="s">
@@ -3387,16 +3412,16 @@
         <v>37</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA6" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AB6" s="12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AC6" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="AD6" s="13"/>
     </row>
@@ -3405,10 +3430,10 @@
         <v>38</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D7" s="14">
         <v>6</v>
@@ -3417,19 +3442,19 @@
         <v>39</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>146</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>147</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>40</v>
@@ -3478,16 +3503,16 @@
         <v>41</v>
       </c>
       <c r="Z7" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA7" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AB7" s="19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AC7" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AD7" s="13"/>
     </row>
@@ -3496,10 +3521,10 @@
         <v>42</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D8" s="6">
         <v>7</v>
@@ -3511,7 +3536,7 @@
         <v>44</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>45</v>
@@ -3520,7 +3545,7 @@
         <v>45</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>31</v>
@@ -3569,16 +3594,16 @@
         <v>46</v>
       </c>
       <c r="Z8" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA8" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AB8" s="20" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AC8" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AD8" s="13"/>
     </row>
@@ -3587,10 +3612,10 @@
         <v>47</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D9" s="14">
         <v>8</v>
@@ -3602,7 +3627,7 @@
         <v>49</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H9" s="7" t="s">
         <v>18</v>
@@ -3611,7 +3636,7 @@
         <v>50</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>36</v>
@@ -3660,28 +3685,28 @@
         <v>51</v>
       </c>
       <c r="Z9" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA9" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AB9" s="12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AC9" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AD9" s="13"/>
     </row>
     <row r="10" spans="1:30" ht="119">
       <c r="A10" s="13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D10" s="6">
         <v>9</v>
@@ -3693,7 +3718,7 @@
         <v>53</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>18</v>
@@ -3702,7 +3727,7 @@
         <v>54</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K10" s="13" t="s">
         <v>19</v>
@@ -3751,28 +3776,28 @@
         <v>55</v>
       </c>
       <c r="Z10" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AA10" s="13" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AB10" s="18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AC10" s="13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="AD10" s="13"/>
     </row>
     <row r="11" spans="1:30" ht="255">
       <c r="A11" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D11" s="14">
         <v>10</v>
@@ -3781,10 +3806,10 @@
         <v>52</v>
       </c>
       <c r="F11" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>192</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>193</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>18</v>
@@ -3793,7 +3818,7 @@
         <v>54</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>56</v>
@@ -3842,28 +3867,28 @@
         <v>57</v>
       </c>
       <c r="Z11" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AA11" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AB11" s="12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AC11" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AD11" s="13"/>
     </row>
     <row r="12" spans="1:30" ht="119">
       <c r="A12" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D12" s="6">
         <v>11</v>
@@ -3875,7 +3900,7 @@
         <v>59</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>60</v>
@@ -3884,7 +3909,7 @@
         <v>61</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K12" s="5" t="s">
         <v>62</v>
@@ -3933,28 +3958,28 @@
         <v>63</v>
       </c>
       <c r="Z12" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA12" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AB12" s="12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AC12" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AD12" s="13"/>
     </row>
     <row r="13" spans="1:30" ht="372">
       <c r="A13" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D13" s="14">
         <v>12</v>
@@ -3966,16 +3991,16 @@
         <v>65</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K13" s="13" t="s">
         <v>40</v>
@@ -4024,28 +4049,28 @@
         <v>66</v>
       </c>
       <c r="Z13" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA13" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AB13" s="18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AC13" s="13" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AD13" s="13"/>
     </row>
     <row r="14" spans="1:30" ht="136">
       <c r="A14" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D14" s="6">
         <v>13</v>
@@ -4054,19 +4079,19 @@
         <v>67</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>18</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K14" s="5" t="s">
         <v>24</v>
@@ -4115,16 +4140,16 @@
         <v>68</v>
       </c>
       <c r="Z14" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AA14" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AB14" s="12" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AC14" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AD14" s="13"/>
     </row>
@@ -4133,17 +4158,17 @@
         <v>76</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="14">
         <v>14</v>
       </c>
       <c r="E15" s="28" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G15" s="13"/>
       <c r="H15" s="15" t="s">
@@ -4173,7 +4198,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T15" s="13"/>
       <c r="U15" s="10"/>
@@ -4187,10 +4212,10 @@
       <c r="AA15" s="13"/>
       <c r="AB15" s="13"/>
       <c r="AC15" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="AD15" s="13" t="s">
         <v>299</v>
-      </c>
-      <c r="AD15" s="13" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="16" spans="1:30" ht="409.6">
@@ -4198,7 +4223,7 @@
         <v>77</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="6">
@@ -4238,7 +4263,7 @@
         <v>0</v>
       </c>
       <c r="S16" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T16" s="5"/>
       <c r="U16" s="10"/>
@@ -4252,10 +4277,10 @@
       <c r="AA16" s="5"/>
       <c r="AB16" s="5"/>
       <c r="AC16" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="AD16" s="13" t="s">
         <v>302</v>
-      </c>
-      <c r="AD16" s="13" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="17" spans="1:30" ht="409.6">
@@ -4263,24 +4288,24 @@
         <v>81</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="14">
         <v>16</v>
       </c>
       <c r="E17" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="F17" s="13" t="s">
         <v>305</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>306</v>
       </c>
       <c r="G17" s="13"/>
       <c r="H17" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="s">
@@ -4303,7 +4328,7 @@
         <v>0</v>
       </c>
       <c r="S17" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T17" s="13"/>
       <c r="U17" s="10"/>
@@ -4317,21 +4342,21 @@
       <c r="AA17" s="13"/>
       <c r="AB17" s="13"/>
       <c r="AC17" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="AD17" s="13" t="s">
         <v>308</v>
-      </c>
-      <c r="AD17" s="13" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="18" spans="1:30" ht="119">
       <c r="A18" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D18" s="6">
         <v>17</v>
@@ -4340,10 +4365,10 @@
         <v>83</v>
       </c>
       <c r="F18" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>199</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>200</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>18</v>
@@ -4352,7 +4377,7 @@
         <v>54</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K18" s="5" t="s">
         <v>84</v>
@@ -4398,19 +4423,19 @@
         <v>46177</v>
       </c>
       <c r="Y18" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="Z18" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA18" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="AB18" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="Z18" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="AA18" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="AB18" s="12" t="s">
-        <v>202</v>
-      </c>
       <c r="AC18" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AD18" s="13"/>
     </row>
@@ -4419,7 +4444,7 @@
         <v>85</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="14">
@@ -4433,14 +4458,14 @@
       </c>
       <c r="G19" s="13"/>
       <c r="H19" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J19" s="13"/>
       <c r="K19" s="13" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L19" s="13" t="s">
         <v>11</v>
@@ -4459,7 +4484,7 @@
         <v>0</v>
       </c>
       <c r="S19" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T19" s="13"/>
       <c r="U19" s="10"/>
@@ -4473,10 +4498,10 @@
       <c r="AA19" s="13"/>
       <c r="AB19" s="13"/>
       <c r="AC19" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="AD19" s="13" t="s">
         <v>312</v>
-      </c>
-      <c r="AD19" s="13" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="20" spans="1:30" ht="409.6">
@@ -4484,7 +4509,7 @@
         <v>88</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="6">
@@ -4524,7 +4549,7 @@
         <v>0</v>
       </c>
       <c r="S20" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T20" s="5"/>
       <c r="U20" s="10"/>
@@ -4538,10 +4563,10 @@
       <c r="AA20" s="5"/>
       <c r="AB20" s="5"/>
       <c r="AC20" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="AD20" s="13" t="s">
         <v>315</v>
-      </c>
-      <c r="AD20" s="13" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="21" spans="1:30" ht="409.6">
@@ -4549,7 +4574,7 @@
         <v>91</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="14">
@@ -4559,14 +4584,14 @@
         <v>92</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="G21" s="13"/>
       <c r="H21" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J21" s="13"/>
       <c r="K21" s="13" t="s">
@@ -4589,7 +4614,7 @@
         <v>0</v>
       </c>
       <c r="S21" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T21" s="13"/>
       <c r="U21" s="10"/>
@@ -4603,10 +4628,10 @@
       <c r="AA21" s="13"/>
       <c r="AB21" s="13"/>
       <c r="AC21" s="13" t="s">
+        <v>317</v>
+      </c>
+      <c r="AD21" s="13" t="s">
         <v>318</v>
-      </c>
-      <c r="AD21" s="13" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="22" spans="1:30" ht="409.6">
@@ -4614,17 +4639,17 @@
         <v>93</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="6">
         <v>21</v>
       </c>
       <c r="E22" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>321</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>322</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="7" t="s">
@@ -4635,10 +4660,10 @@
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="L22" s="5" t="s">
         <v>323</v>
-      </c>
-      <c r="L22" s="5" t="s">
-        <v>324</v>
       </c>
       <c r="M22" s="7">
         <v>200</v>
@@ -4654,7 +4679,7 @@
         <v>0</v>
       </c>
       <c r="S22" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T22" s="5"/>
       <c r="U22" s="10"/>
@@ -4668,10 +4693,10 @@
       <c r="AA22" s="5"/>
       <c r="AB22" s="5"/>
       <c r="AC22" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="AD22" s="13" t="s">
         <v>325</v>
-      </c>
-      <c r="AD22" s="13" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="23" spans="1:30" ht="409.6">
@@ -4679,7 +4704,7 @@
         <v>95</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="14">
@@ -4719,7 +4744,7 @@
         <v>0</v>
       </c>
       <c r="S23" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T23" s="13"/>
       <c r="U23" s="10"/>
@@ -4733,10 +4758,10 @@
       <c r="AA23" s="13"/>
       <c r="AB23" s="13"/>
       <c r="AC23" s="13" t="s">
+        <v>327</v>
+      </c>
+      <c r="AD23" s="13" t="s">
         <v>328</v>
-      </c>
-      <c r="AD23" s="13" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="24" spans="1:30" ht="409.6">
@@ -4744,7 +4769,7 @@
         <v>98</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="6">
@@ -4758,10 +4783,10 @@
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="5" t="s">
@@ -4784,7 +4809,7 @@
         <v>0</v>
       </c>
       <c r="S24" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T24" s="5"/>
       <c r="U24" s="10"/>
@@ -4798,10 +4823,10 @@
       <c r="AA24" s="5"/>
       <c r="AB24" s="5"/>
       <c r="AC24" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="AD24" s="13" t="s">
         <v>331</v>
-      </c>
-      <c r="AD24" s="13" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="25" spans="1:30" ht="409.6">
@@ -4809,14 +4834,14 @@
         <v>101</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C25" s="13"/>
       <c r="D25" s="14">
         <v>24</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>102</v>
@@ -4849,7 +4874,7 @@
         <v>0</v>
       </c>
       <c r="S25" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T25" s="13"/>
       <c r="U25" s="10"/>
@@ -4863,21 +4888,21 @@
       <c r="AA25" s="13"/>
       <c r="AB25" s="13"/>
       <c r="AC25" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="AD25" s="13" t="s">
         <v>335</v>
-      </c>
-      <c r="AD25" s="13" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="26" spans="1:30" ht="289">
       <c r="A26" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D26" s="6">
         <v>25</v>
@@ -4889,16 +4914,16 @@
         <v>104</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="K26" s="5" t="s">
         <v>82</v>
@@ -4944,31 +4969,31 @@
         <v>46224</v>
       </c>
       <c r="Y26" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="Z26" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AA26" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AB26" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AC26" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="AD26" s="13"/>
     </row>
     <row r="27" spans="1:30" ht="255">
       <c r="A27" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D27" s="14">
         <v>26</v>
@@ -4977,10 +5002,10 @@
         <v>105</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>18</v>
@@ -4989,10 +5014,10 @@
         <v>54</v>
       </c>
       <c r="J27" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K27" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L27" s="13" t="s">
         <v>20</v>
@@ -5035,19 +5060,19 @@
         <v>46234</v>
       </c>
       <c r="Y27" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="Z27" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AA27" s="13" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AB27" s="21" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="AC27" s="13" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="AD27" s="13"/>
     </row>
@@ -5056,7 +5081,7 @@
         <v>106</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="6">
@@ -5096,7 +5121,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T28" s="5"/>
       <c r="U28" s="10"/>
@@ -5110,31 +5135,31 @@
       <c r="AA28" s="5"/>
       <c r="AB28" s="5"/>
       <c r="AC28" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD28" s="13" t="s">
         <v>338</v>
-      </c>
-      <c r="AD28" s="13" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="29" spans="1:30" ht="289">
       <c r="A29" s="13" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C29" s="13"/>
       <c r="D29" s="14">
         <v>28</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="F29" s="13" t="s">
         <v>108</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>18</v>
@@ -5143,7 +5168,7 @@
         <v>54</v>
       </c>
       <c r="J29" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K29" s="13" t="s">
         <v>56</v>
@@ -5189,19 +5214,19 @@
         <v>46232</v>
       </c>
       <c r="Y29" s="13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Z29" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AA29" s="13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AB29" s="18" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="AC29" s="13" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="AD29" s="13"/>
     </row>
@@ -5210,10 +5235,10 @@
         <v>109</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D30" s="6">
         <v>29</v>
@@ -5225,16 +5250,16 @@
         <v>111</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H30" s="7" t="s">
         <v>18</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>24</v>
@@ -5281,19 +5306,19 @@
         <v>46233</v>
       </c>
       <c r="Y30" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="Z30" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA30" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="AB30" s="12" t="s">
         <v>277</v>
       </c>
-      <c r="Z30" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="AA30" s="5" t="s">
-        <v>280</v>
-      </c>
-      <c r="AB30" s="12" t="s">
+      <c r="AC30" s="5" t="s">
         <v>278</v>
-      </c>
-      <c r="AC30" s="5" t="s">
-        <v>279</v>
       </c>
       <c r="AD30" s="13"/>
     </row>
@@ -5302,24 +5327,24 @@
         <v>112</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="14">
         <v>30</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F31" s="22" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J31" s="5"/>
       <c r="K31" s="5" t="s">
@@ -5342,7 +5367,7 @@
         <v>0</v>
       </c>
       <c r="S31" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T31" s="5"/>
       <c r="U31" s="10"/>
@@ -5356,21 +5381,21 @@
       <c r="AA31" s="5"/>
       <c r="AB31" s="5"/>
       <c r="AC31" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="AD31" s="13" t="s">
         <v>342</v>
-      </c>
-      <c r="AD31" s="13" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="32" spans="1:30" ht="119">
       <c r="A32" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>159</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>160</v>
       </c>
       <c r="D32" s="6">
         <v>31</v>
@@ -5382,7 +5407,7 @@
         <v>74</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H32" s="7" t="s">
         <v>18</v>
@@ -5391,7 +5416,7 @@
         <v>50</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>24</v>
@@ -5440,16 +5465,16 @@
         <v>75</v>
       </c>
       <c r="Z32" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AA32" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AB32" s="12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AC32" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AD32" s="13"/>
     </row>
@@ -5510,46 +5535,46 @@
       <c r="AA33" s="13"/>
       <c r="AB33" s="13"/>
       <c r="AC33" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AD33" s="13"/>
     </row>
     <row r="34" spans="1:30" ht="136">
       <c r="A34" s="13" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D34" s="14">
         <v>33</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="H34" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I34" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J34" s="13" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="K34" s="13" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="M34" s="29">
         <v>365.39866899999998</v>
@@ -5589,19 +5614,19 @@
         <v>46260</v>
       </c>
       <c r="Y34" s="13" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="Z34" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AA34" s="13" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="AB34" s="13" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="AC34" s="13" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="AD34" s="13"/>
     </row>
@@ -5610,7 +5635,7 @@
         <v>117</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C35" s="13"/>
       <c r="D35" s="14">
@@ -5650,7 +5675,7 @@
         <v>0</v>
       </c>
       <c r="S35" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T35" s="13"/>
       <c r="U35" s="10"/>
@@ -5664,20 +5689,22 @@
       <c r="AA35" s="13"/>
       <c r="AB35" s="13"/>
       <c r="AC35" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="AD35" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="AD35" s="13" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="36" spans="1:30" ht="409.6">
+    </row>
+    <row r="36" spans="1:30" ht="102">
       <c r="A36" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C36" s="5"/>
+        <v>478</v>
+      </c>
+      <c r="B36" s="31" t="s">
+        <v>479</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>147</v>
+      </c>
       <c r="D36" s="6">
         <v>35</v>
       </c>
@@ -5685,89 +5712,113 @@
         <v>103</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="G36" s="5"/>
+        <v>119</v>
+      </c>
+      <c r="G36" s="31" t="s">
+        <v>480</v>
+      </c>
       <c r="H36" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="I36" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="J36" s="5"/>
+        <v>143</v>
+      </c>
+      <c r="I36" s="31" t="s">
+        <v>481</v>
+      </c>
+      <c r="J36" s="31" t="s">
+        <v>481</v>
+      </c>
       <c r="K36" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="L36" s="5" t="s">
-        <v>32</v>
+      <c r="L36" s="31" t="s">
+        <v>482</v>
       </c>
       <c r="M36" s="7">
-        <v>2400</v>
+        <v>2693</v>
       </c>
       <c r="N36" s="7">
-        <v>2400</v>
-      </c>
-      <c r="O36" s="7"/>
-      <c r="P36" s="8"/>
-      <c r="Q36" s="8"/>
+        <v>2693</v>
+      </c>
+      <c r="O36" s="7">
+        <v>2693</v>
+      </c>
+      <c r="P36" s="16">
+        <v>785</v>
+      </c>
+      <c r="Q36" s="16">
+        <v>881</v>
+      </c>
       <c r="R36" s="9">
-        <f>SUM(Tabla22[[#This Row],[inversion_activos_computables_comprometida_anio_1_mill_usd]:[inversion_activos_computables_comprometida_anio_2_mill_usd]])</f>
-        <v>0</v>
+        <f>SUM([1]!Tabla22[[#This Row],[inversion_activos_computables_comprometida_anio_1_mill_usd]:[inversion_activos_computables_comprometida_anio_2_mill_usd]])</f>
+        <v>1666</v>
       </c>
       <c r="S36" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="T36" s="5"/>
-      <c r="U36" s="10"/>
+        <v>14</v>
+      </c>
+      <c r="T36" s="5">
+        <v>12500</v>
+      </c>
+      <c r="U36" s="30">
+        <v>47453</v>
+      </c>
       <c r="V36" s="11">
-        <v>46136</v>
-      </c>
-      <c r="W36" s="11"/>
-      <c r="X36" s="11"/>
-      <c r="Y36" s="5"/>
-      <c r="Z36" s="5"/>
-      <c r="AA36" s="5"/>
-      <c r="AB36" s="5"/>
+        <v>46237</v>
+      </c>
+      <c r="W36" s="11">
+        <v>46237</v>
+      </c>
+      <c r="X36" s="11">
+        <v>46272</v>
+      </c>
+      <c r="Y36" s="5" t="s">
+        <v>483</v>
+      </c>
+      <c r="Z36" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA36" s="31" t="s">
+        <v>484</v>
+      </c>
+      <c r="AB36" s="32" t="s">
+        <v>485</v>
+      </c>
       <c r="AC36" s="5" t="s">
-        <v>348</v>
-      </c>
-      <c r="AD36" s="13" t="s">
-        <v>349</v>
-      </c>
+        <v>486</v>
+      </c>
+      <c r="AD36" s="13"/>
     </row>
     <row r="37" spans="1:30" ht="204">
       <c r="A37" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D37" s="14">
         <v>36</v>
       </c>
       <c r="E37" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="F37" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="F37" s="13" t="s">
-        <v>122</v>
-      </c>
       <c r="G37" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="I37" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="J37" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="K37" s="13" t="s">
         <v>241</v>
-      </c>
-      <c r="H37" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="I37" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="J37" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="K37" s="13" t="s">
-        <v>242</v>
       </c>
       <c r="L37" s="13" t="s">
         <v>11</v>
@@ -5810,19 +5861,19 @@
         <v>46198</v>
       </c>
       <c r="Y37" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="Z37" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA37" s="13" t="s">
+        <v>370</v>
+      </c>
+      <c r="AB37" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="Z37" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="AA37" s="13" t="s">
-        <v>375</v>
-      </c>
-      <c r="AB37" s="21" t="s">
+      <c r="AC37" s="13" t="s">
         <v>244</v>
-      </c>
-      <c r="AC37" s="13" t="s">
-        <v>245</v>
       </c>
       <c r="AD37" s="13"/>
     </row>
@@ -5831,10 +5882,10 @@
         <v>69</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D38" s="6">
         <v>37</v>
@@ -5846,7 +5897,7 @@
         <v>71</v>
       </c>
       <c r="G38" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H38" s="15" t="s">
         <v>18</v>
@@ -5855,7 +5906,7 @@
         <v>54</v>
       </c>
       <c r="J38" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K38" s="13" t="s">
         <v>56</v>
@@ -5904,35 +5955,35 @@
         <v>72</v>
       </c>
       <c r="Z38" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA38" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AB38" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC38" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AD38" s="13"/>
     </row>
     <row r="39" spans="1:30" ht="409.6">
       <c r="A39" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="14">
         <v>38</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="G39" s="5"/>
       <c r="H39" s="7" t="s">
@@ -5962,7 +6013,7 @@
         <v>0</v>
       </c>
       <c r="S39" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T39" s="5"/>
       <c r="U39" s="10"/>
@@ -5976,35 +6027,35 @@
       <c r="AA39" s="5"/>
       <c r="AB39" s="5"/>
       <c r="AC39" s="5" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="AD39" s="13" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
     </row>
     <row r="40" spans="1:30" ht="409.6">
       <c r="A40" s="13" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="6">
         <v>39</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="G40" s="13"/>
       <c r="H40" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I40" s="13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J40" s="13"/>
       <c r="K40" s="13" t="s">
@@ -6027,7 +6078,7 @@
         <v>0</v>
       </c>
       <c r="S40" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T40" s="13"/>
       <c r="U40" s="10"/>
@@ -6041,35 +6092,35 @@
       <c r="AA40" s="13"/>
       <c r="AB40" s="13"/>
       <c r="AC40" s="13" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="AD40" s="13" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="41" spans="1:30" ht="409.6">
       <c r="A41" s="13" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="C41" s="13"/>
       <c r="D41" s="14">
         <v>40</v>
       </c>
       <c r="E41" s="15" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="G41" s="13"/>
       <c r="H41" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I41" s="13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J41" s="13"/>
       <c r="K41" s="13" t="s">
@@ -6092,7 +6143,7 @@
         <v>0</v>
       </c>
       <c r="S41" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T41" s="17"/>
       <c r="U41" s="10"/>
@@ -6106,39 +6157,39 @@
       <c r="AA41" s="13"/>
       <c r="AB41" s="13"/>
       <c r="AC41" s="13" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="AD41" s="18" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="42" spans="1:30" ht="409.6">
       <c r="A42" s="13" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="14">
         <v>41</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="G42" s="13"/>
       <c r="H42" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I42" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J42" s="13"/>
       <c r="K42" s="13" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L42" s="13" t="s">
         <v>11</v>
@@ -6155,7 +6206,7 @@
         <v>0</v>
       </c>
       <c r="S42" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T42" s="15"/>
       <c r="U42" s="10"/>
@@ -6169,10 +6220,10 @@
       <c r="AA42" s="13"/>
       <c r="AB42" s="13"/>
       <c r="AC42" s="13" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="AD42" s="13" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
     </row>
     <row r="43" spans="1:30">
@@ -6232,12 +6283,13 @@
     <hyperlink ref="AD41" r:id="rId20" xr:uid="{8B349C04-C00D-AF45-A235-16E6BEF78B40}"/>
     <hyperlink ref="AB27" r:id="rId21" xr:uid="{C5A97FE8-FC03-4B41-86D8-2D3DFD0E915C}"/>
     <hyperlink ref="AB37" r:id="rId22" xr:uid="{95B4063F-E390-2F4C-97F4-22710E08828D}"/>
+    <hyperlink ref="AB36" r:id="rId23" xr:uid="{9B51BCFC-E252-834C-AFEB-4F698D772E88}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId23"/>
-  <legacyDrawing r:id="rId24"/>
+  <drawing r:id="rId24"/>
+  <legacyDrawing r:id="rId25"/>
   <tableParts count="1">
-    <tablePart r:id="rId25"/>
+    <tablePart r:id="rId26"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6257,22 +6309,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="24" t="s">
+        <v>389</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>463</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>464</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>392</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>393</v>
+      </c>
+      <c r="F1" s="24" t="s">
         <v>394</v>
-      </c>
-      <c r="B1" s="24" t="s">
-        <v>468</v>
-      </c>
-      <c r="C1" s="24" t="s">
-        <v>469</v>
-      </c>
-      <c r="D1" s="24" t="s">
-        <v>397</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>398</v>
-      </c>
-      <c r="F1" s="24" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16">
@@ -6280,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16">
@@ -6300,19 +6352,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16">
@@ -6320,19 +6372,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16">
@@ -6343,16 +6395,16 @@
         <v>0</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16">
@@ -6363,16 +6415,16 @@
         <v>1</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16">
@@ -6380,19 +6432,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16">
@@ -6400,19 +6452,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16">
@@ -6423,16 +6475,16 @@
         <v>2</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16">
@@ -6443,16 +6495,16 @@
         <v>3</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16">
@@ -6460,19 +6512,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16">
@@ -6483,16 +6535,16 @@
         <v>4</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16">
@@ -6503,16 +6555,16 @@
         <v>5</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16">
@@ -6520,19 +6572,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16">
@@ -6540,19 +6592,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16">
@@ -6560,19 +6612,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E16" s="23" t="s">
+        <v>425</v>
+      </c>
+      <c r="F16" s="23" t="s">
         <v>430</v>
-      </c>
-      <c r="F16" s="23" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="16">
@@ -6580,19 +6632,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="16">
@@ -6600,19 +6652,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="32">
@@ -6620,19 +6672,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="16">
@@ -6640,19 +6692,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F20" s="23" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16">
@@ -6660,19 +6712,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="16">
@@ -6680,19 +6732,19 @@
         <v>21</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="16">
@@ -6703,16 +6755,16 @@
         <v>6</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="16">
@@ -6720,19 +6772,19 @@
         <v>23</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="D24" s="23" t="s">
+        <v>442</v>
+      </c>
+      <c r="E24" s="23" t="s">
+        <v>442</v>
+      </c>
+      <c r="F24" s="23" t="s">
         <v>447</v>
-      </c>
-      <c r="E24" s="23" t="s">
-        <v>447</v>
-      </c>
-      <c r="F24" s="23" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="16">
@@ -6740,19 +6792,19 @@
         <v>24</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="16">
@@ -6763,16 +6815,16 @@
         <v>7</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="32">
@@ -6780,19 +6832,19 @@
         <v>26</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="16">
@@ -6800,19 +6852,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="16">
@@ -6820,19 +6872,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="16">
@@ -6840,19 +6892,19 @@
         <v>29</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="16">
@@ -6860,19 +6912,19 @@
         <v>30</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -6887,13 +6939,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="60">
       <c r="A1" s="26" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -6901,10 +6953,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="45">
@@ -6912,10 +6964,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="105">
@@ -6923,10 +6975,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -6956,10 +7008,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -6967,10 +7019,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -7000,10 +7052,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -7033,10 +7085,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="60">
@@ -7044,10 +7096,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="60">
@@ -7055,10 +7107,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="90">
@@ -7066,10 +7118,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="90">
@@ -7077,10 +7129,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="90">
@@ -7088,10 +7140,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="45">
@@ -7099,10 +7151,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="60">
@@ -7110,10 +7162,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="75">
@@ -7121,10 +7173,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30">
@@ -7143,10 +7195,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30">
@@ -7154,10 +7206,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="30">
@@ -7176,10 +7228,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="27" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="60">
@@ -7187,10 +7239,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="27" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -7198,10 +7250,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -7209,10 +7261,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="27" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="30">
@@ -7220,10 +7272,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualizacion fecha de presentacion sal de oro
</commit_message>
<xml_diff>
--- a/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
+++ b/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/base de datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217E0B12-3668-5849-9BD1-32C9FCFD18AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F8D117A-E4BA-A64B-83DE-1C65C25B9F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="35760" yWindow="600" windowWidth="33020" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5190,7 +5190,7 @@
         <v>47330</v>
       </c>
       <c r="V27" s="24">
-        <v>45595</v>
+        <v>45978</v>
       </c>
       <c r="W27" s="24">
         <v>46185</v>

</xml_diff>